<commit_message>
Add example Data and Template files
</commit_message>
<xml_diff>
--- a/Data/interns.xlsx
+++ b/Data/interns.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interns" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,50 +429,30 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Roles</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Duty</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Company Name</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Roles</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Duty</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Company Name</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Intern ID</t>
-        </is>
-      </c>
       <c r="H1" t="inlineStr">
-        <is>
-          <t>Duration</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Mode</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Stipend</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Commitment</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
         <is>
           <t>Intern Id</t>
         </is>
@@ -481,83 +461,61 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yuvraj </t>
+          <t>Alice Example</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>yuvrajsinghbhadouria19@gmail.com</t>
+          <t>alice@example.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Sent</t>
+          <t>Technical</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Technical</t>
+          <t>Backend development</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cyber </t>
+          <t>8 weeks</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Connectbiopay</t>
+          <t>Biopay</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>2 Month</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Online</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>10000</v>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>20hrs/week</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>CONNYU540</t>
-        </is>
-      </c>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>raj</t>
+          <t>Bob Sample</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>rajsinghb532@gmail.com</t>
+          <t>bob@example.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Sent</t>
+          <t>Non-Technical</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Non technical</t>
+          <t>Marketing support</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Hr</t>
+          <t>6 weeks</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -566,201 +524,7 @@
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>2 Month</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Hybrid</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>10000</v>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>20hrs/week</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>BIOPRA875</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Yuvraj Singh</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Yuvraj.14336@stu.upes.ac.in</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Sent</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Non technical</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>PR</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Saas</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>3 Month</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Offline</t>
-        </is>
-      </c>
-      <c r="J4" t="n">
-        <v>10000</v>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>16hrs/week</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>SAASYU911</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Sangeeta</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>sangeetabhadouria983@gmail.com</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Sent</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Non technical</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Head</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Connectbiopay</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>2 Months</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Offline</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Unpaid</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>10hrs/week</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>CONNSA531</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Anmol</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Anmolsingh260308@gmail.com</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Sent</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Non technical</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>PR</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Connectbiopay</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>2 months</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>offline</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>unpaid</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>10hrs/week</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>CONNAN545</t>
-        </is>
-      </c>
+      <c r="H3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>